<commit_message>
Main updates to CH card v6
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v6/CH_Card/CH_Card_BOM_digikey.xlsx
+++ b/Lasser_Driver_v6/CH_Card/CH_Card_BOM_digikey.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>CH_Card U26,U104,U105</t>
+          <t>CH_Card U26,U104,U105,U108</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -607,13 +607,13 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>SPDT analog switch (lock switch + ERR/MOD channel muxes)</t>
+          <t>SPDT analog switch (lock switch, ERR/MOD channel muxes, TEC 0 A safe-state)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CH_Card U17,U19,U22,U24</t>
+          <t>CH_Card U17,U19,U22,U24,U106</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -642,13 +642,13 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Precision op-amp 36V (VZERO buf, TEC err, laser set, summing) - SEE NOTE: symbol unit renumber to DBV</t>
+          <t>Precision op-amp 36V (VZERO buf, TEC err, laser set, summing, leg-1 drive inverter) - SEE NOTE: symbol unit renumber to DBV</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CH_Card U21</t>
+          <t>CH_Card U21,U107</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Power op-amp 60V 200mA w/ thermal flag (H-bridge gate driver)</t>
+          <t>Power op-amp 60V 200mA w/ thermal flag (H-bridge gate drivers: U21 = leg 2, U107 = leg 1)</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>CH_Card D22</t>
+          <t>CH_Card D22,D23</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Schottky 100V 75mA laser reverse protect (SUB for BAT54: no SOD-123 variant)</t>
+          <t>Schottky 100V 75mA - D22 laser reverse protect, D23 OPA551 flag clamp to 3V3</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R49,R79,R92,R96,R115,R120,R121,R122,R123,R124,R125,R127,R128,R129,R_f1,R_f2</t>
+          <t>CH_Card R79,R92,R115,R120,R121,R122,R123,R124,R125,R127,R128,R129,R130,R131,R133,R_f1,R_f2</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1138,7 +1138,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R48,R116,R126</t>
+          <t>CH_Card R48,R116,R126,R132</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1173,7 +1173,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R56,R57,R58,R59,R69,R70,R75</t>
+          <t>CH_Card R69,R70,R75</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Res 47R 1% (gate resistors + NTC/monitor line protection)</t>
+          <t>Res 47R 1% (NTC + monitor line protection; gate drive moved to the 470R line)</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R77</t>
+          <t>CH_Card R77,R117</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Res 2k 1% (trim)</t>
+          <t>Res 2k 1% (R77 RF trim; R117 VZERO trim series - was 4.99k, in series with R43 20k into VZERO_SET so it sets the DAC trim span)</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R44,R117,R118,R119</t>
+          <t>CH_Card R44,R118,R119</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1517,67 +1517,67 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Res 4.99k 0.1% (TEC scaler top, VZERO trim, ADC prot) - ERA-6AEB4991V 0 stock</t>
+          <t>Res 4.99k 0.1% (TEC scaler top, ADC prot) - ERA-6AEB4991V 0 stock</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>TNPW08051K00BEEA</t>
+          <t>CL21B104KBCNNNC</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R67</t>
+          <t>CH_Card C65,C66,C116,C117,C118,C122,C123,C130,C131,C132,C133,C134,C135,C136,C137,C138,C139,C140,C141,C142,C143,C144,C145,C146,C147,C148,C149,C152,C153,C155,C156,C158,C161,C164,C165,C166,C167,C168,C169,C170,C171,C172,C173,C174,C_NTC1</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>1k 0.1%</t>
+          <t>100nF</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>R_0805</t>
+          <t>C_0805</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Res 1k 0.1% (laser scaler bottom) - ERA-6AEB102V 0 stock</t>
+          <t>MLCC 100nF 50V X7R (decoupling bank + misc; same as pm1p8V)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>CL21B104KBCNNNC</t>
+          <t>C0805C105K5RACTU</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>KEMET</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C65,C66,C_NTC1,C116,C117,C118,C122,C123,C130,C131,C132,C133,C134,C135,C136,C137,C138,C139,C140,C141,C142,C143,C144,C145,C146,C147,C148,C149,C152,C153,C155,C156,C158,C161,C164,C165,C166</t>
+          <t>CH_Card C113,C114</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>100nF</t>
+          <t>1uF</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1587,17 +1587,17 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>MLCC 100nF 50V X7R (decoupling bank + misc; same as pm1p8V)</t>
+          <t>MLCC 1uF 50V X7R (DAC output filters; same as pm1p8V)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>C0805C105K5RACTU</t>
+          <t>C0805C106K3PACTU</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -1607,12 +1607,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C113,C114</t>
+          <t>CH_Card C115,C121,C150,C151,C154,C157,C160,C163</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>1uF</t>
+          <t>10uF</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1622,42 +1622,42 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>MLCC 1uF 50V X7R (DAC output filters; same as pm1p8V)</t>
+          <t>MLCC 10uF 25V X5R (rail bulk; same as pm1p8V)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>C0805C106K3PACTU</t>
+          <t>1210YD107MAT2A</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>KEMET</t>
+          <t>KYOCERA AVX</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C115,C121,C150,C151,C154,C157,C160,C163</t>
+          <t>CH_Card C159,C162</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>10uF</t>
+          <t>100uF</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>C_0805</t>
+          <t>C_1210</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>MLCC 10uF 25V X5R (rail bulk; same as pm1p8V)</t>
+          <t>MLCC 100uF 16V X5R (+/-6V_TEC bulk; same as pm1p8V)</t>
         </is>
       </c>
     </row>
@@ -1667,57 +1667,57 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>1210YD107MAT2A</t>
+          <t>CL21B103KBANNNC</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>KYOCERA AVX</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C159,C162</t>
+          <t>CH_Card C119,C120</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>100uF</t>
+          <t>10nF</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>C_1210</t>
+          <t>C_0805</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>MLCC 100uF 16V X5R (+/-6V_TEC bulk; same as pm1p8V)</t>
+          <t>MLCC 10nF 50V X7R (ADC input filters)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>CL21B103KBANNNC</t>
+          <t>C0805C103J5GACTU</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>KEMET</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C119,C120</t>
+          <t>CH_Card C70</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>10nF</t>
+          <t>10nF C0G</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>MLCC 10nF 50V X7R (ADC input filters)</t>
+          <t>MLCC 10nF 50V C0G (laser filter)</t>
         </is>
       </c>
     </row>
@@ -1737,22 +1737,22 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>C0805C103J5GACTU</t>
+          <t>CL21B102KBANNNC</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>KEMET</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C70</t>
+          <t>CH_Card C76</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>10nF C0G</t>
+          <t>1nF</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>MLCC 10nF 50V C0G (laser filter)</t>
+          <t>MLCC 1nF 50V X7R (lock integrator Ci)</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>CL21B102KBANNNC</t>
+          <t>CL21C101JBANNNC</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C76</t>
+          <t>CH_Card C68</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>1nF</t>
+          <t>100pF NP0</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1797,77 +1797,77 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>MLCC 1nF 50V X7R (lock integrator Ci)</t>
+          <t>MLCC 100pF 50V C0G (comp)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>CL21C101JBANNNC</t>
+          <t>GRM1555C1H2R2CA01D</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>Murata Electronics</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C68</t>
+          <t>CH_Card C_f1,C_f2</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>100pF NP0</t>
+          <t>2.2pF</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>C_0805</t>
+          <t>C_0402</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>MLCC 100pF 50V C0G (comp)</t>
+          <t>MLCC 2.2pF 50V C0G 0402 (TIA feedback; CL05C2R2CB5NNNC obsolete)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>GRM1555C1H2R2CA01D</t>
+          <t>374144-E</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Murata Electronics</t>
+          <t>TE Connectivity AMP</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>CH_Card C_f1,C_f2</t>
+          <t>CH_Card J1</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>2.2pF</t>
+          <t>DIN41612 M 3x8+8</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>C_0402</t>
+          <t>DIN41612_M_Power_Male</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>MLCC 2.2pF 50V C0G 0402 (TIA feedback; CL05C2R2CB5NNNC obsolete)</t>
+          <t>DIN41612 Type M 24sig+8pwr R/A male (same as pm6V/pm1p8V) - 0 STOCK, check lead time</t>
         </is>
       </c>
     </row>
@@ -1877,67 +1877,67 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>374144-E</t>
+          <t>61301421121</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>TE Connectivity AMP</t>
+          <t>Würth Elektronik</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>CH_Card J1</t>
+          <t>CH_Card J_BTF1</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>DIN41612 M 3x8+8</t>
+          <t>2x7 pin header</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>DIN41612_M_Power_Male</t>
+          <t>PinHeader_2x07_P2.54mm_Vertical</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>DIN41612 Type M 24sig+8pwr R/A male (same as pm6V/pm1p8V) - 0 STOCK, check lead time</t>
+          <t>Würth WR-PHD 2.54mm 2x7 male pin header - board side of the off-board laser-head harness; same connector family as the LDM-BUTTERFLY mount socket (Würth 61301421821). Wire assembly (cable) sourced separately - spec 24AWG for the TEC pair.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>61301421121</t>
+          <t>61300211121</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Würth Elektronik</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>CH_Card J_BTF1</t>
+          <t>CH_Card JP101,JP102,JP103</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>2x7 pin header</t>
+          <t>1x2 header</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>PinHeader_2x07_P2.54mm_Vertical</t>
+          <t>PinHeader_1x02</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Würth WR-PHD 2.54mm 2x7 male pin header - board side of the off-board laser-head harness; same connector family as the LDM-BUTTERFLY mount socket (Würth 61301421821). Wire assembly (cable) sourced separately - spec 24AWG for the TEC pair.</t>
+          <t>Pin header 1x2 2.54mm (GA address jumpers)</t>
         </is>
       </c>
     </row>
@@ -1947,67 +1947,67 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>61300211121</t>
+          <t>SPC02SYAN</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Wurth Elektronik</t>
+          <t>Sullins Connector</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>CH_Card JP101,JP102,JP103</t>
+          <t>CH_Card JP101-103 shunts</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>1x2 header</t>
+          <t>shunt</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>PinHeader_1x02</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Pin header 1x2 2.54mm (GA address jumpers)</t>
+          <t>Shorting jumper 2.54mm gold (fit = address bit 0)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>SPC02SYAN</t>
+          <t>657-10ABPE</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Sullins Connector</t>
+          <t>Wakefield Thermal Solutions</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>CH_Card JP101-103 shunts</t>
+          <t>CH_Card HS1,HS2,HS3,HS4</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>shunt</t>
+          <t>Heatsink TO-220 vert 1in</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TO-220-3_Vertical_HS657</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Shorting jumper 2.54mm gold (fit = address bit 0)</t>
+          <t>Vert board-mount heatsink 657-series 25.4mm, 6.8C/W nat (TEC H-bridge Q13/Q14/Q17/Q18; same as pm6V)</t>
         </is>
       </c>
     </row>
@@ -2017,32 +2017,32 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>657-10ABPE</t>
+          <t>4880G</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Wakefield Thermal Solutions</t>
+          <t>Boyd</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>CH_Card HS1,HS2,HS3,HS4</t>
+          <t>CH_Card Q13,Q14,Q17,Q18 (TO-220 iso)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Heatsink TO-220 vert 1in</t>
+          <t>TO-220 mount kit</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>TO-220-3_Vertical_HS657</t>
+          <t>Hardware (off-PCB)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Vert board-mount heatsink 657-series 25.4mm, 6.8C/W nat (TEC H-bridge Q13/Q14/Q17/Q18; same as pm6V)</t>
+          <t>Insulator+shoulder washer kit; isolates FET tab from heatsink (tabs are live: +6V_TEC / bridge outputs)</t>
         </is>
       </c>
     </row>
@@ -2052,22 +2052,22 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>4880G</t>
+          <t>PMSSS 440 0050 PH</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Boyd</t>
+          <t>B&amp;F Fastener Supply</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>CH_Card Q13,Q14,Q17,Q18 (TO-220 iso)</t>
+          <t>CH_Card Q13-Q18 heatsink mount</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>TO-220 mount kit</t>
+          <t>#4-40 x 1/2in screw</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Insulator+shoulder washer kit; isolates FET tab from heatsink (tabs are live: +6V_TEC / bridge outputs)</t>
+          <t>SS pan-head machine screw #4-40 x 1/2in (FET to 657 web)</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>PMSSS 440 0050 PH</t>
+          <t>FWSS 004</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>#4-40 x 1/2in screw</t>
+          <t>#4 flat washer</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>SS pan-head machine screw #4-40 x 1/2in (FET to 657 web)</t>
+          <t>SS #4 flat washer, nut side</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>FWSS 004</t>
+          <t>INTLWZ 004</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>#4 flat washer</t>
+          <t>#4 int-tooth lock washer</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>SS #4 flat washer, nut side</t>
+          <t>Internal-tooth lock washer #4 (anti-rotation)</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>INTLWZ 004</t>
+          <t>HNZ 440</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>#4 int-tooth lock washer</t>
+          <t>#4-40 hex nut</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2182,42 +2182,42 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Internal-tooth lock washer #4 (anti-rotation)</t>
+          <t>#4-40 hex nut, zinc-plated steel</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>HNZ 440</t>
+          <t>WSL2512R0100FEA</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>B&amp;F Fastener Supply</t>
+          <t>Vishay Dale</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>CH_Card Q13-Q18 heatsink mount</t>
+          <t>CH_Card R68,R76</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>#4-40 hex nut</t>
+          <t>10mR link</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Hardware (off-PCB)</t>
+          <t>R_2512</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>#4-40 hex nut, zinc-plated steel</t>
+          <t>0.01R 1% 1W 2512 - TEC drive links to butterfly (was 47R: blocked TEC current)</t>
         </is>
       </c>
     </row>
@@ -2227,67 +2227,242 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>WSL2512R0100FEA</t>
+          <t>RC0805JR-070RL</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Vishay Dale</t>
+          <t>YAGEO</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>CH_Card R68,R76</t>
+          <t>CH_Card R73,R74</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>10mR link</t>
+          <t>0R link</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>R_2512</t>
+          <t>R_0805</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>0.01R 1% 1W 2512 - TEC drive links to butterfly (was 47R: blocked TEC current)</t>
+          <t>0R jumper - laser CHIP+/- links (was 47R: no laser headroom)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>RC0805JR-070RL</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="A53" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ERA-6AEB9090V</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Panasonic Industry</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CH_Card R67</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>909R 0.1%</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>R_0805</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Res 909R 0.1% (laser scaler BOTTOM, to GND) - sets DAC full scale 90.5 mA</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>RC0805FR-077M5L</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>YAGEO</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>CH_Card R73,R74</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>0R link</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CH_Card R96</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>7.5M</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
         <is>
           <t>R_0805</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>0R jumper - laser CHIP+/- links (was 47R: no laser headroom)</t>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Res 7.5M 1% (PDH servo injection into the laser setpoint; 0.483 mA/V)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>1</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>RC0805JR-0715ML</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>CH_Card R134</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>15M</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>R_0805</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Res 15M 5% (cancels U24's 2.500V VREF_MID pedestal via -5V; exact 2:1 with R96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>1</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>RC0805FR-0733KL</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>CH_Card R49</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>33k</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>R_0805</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Res 33k 1% (OPA551 flag PULL-DOWN: flag is a current source, 80uA min -&gt; 2.64V &gt; VIH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>4</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>RC0805FR-07470RL</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>CH_Card R56,R57,R58,R59</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>470R</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>R_0805</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Res 470R 1% gate drive - 47R let a saturated buffer pull 353 mA from a 200 mA OPA551</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>1</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>RC0805FR-07100KL</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>CH_Card R78</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>100k</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>R_0805</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Res 100k 1% - DC bleed on the MOD injection island (C66-R77-C70); was missing from the BOM</t>
         </is>
       </c>
     </row>

</xml_diff>